<commit_message>
handling author complex data structure
</commit_message>
<xml_diff>
--- a/citations/test_df.xlsx
+++ b/citations/test_df.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AQ2"/>
+  <dimension ref="A1:AP2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -547,35 +547,28 @@
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>topics</t>
+          <t>topic</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>topic</t>
+          <t>subfield</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>subfield</t>
+          <t>field</t>
         </is>
       </c>
       <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
+      <c r="A2">
+        <v>2023</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -592,11 +585,6 @@
           <t>The Glasgow Climate Conference (COP26)</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>https://openalex.org/A5087355631: Mitchell Lennan: https://orcid.org/0000-0003-4744-4496: first: FALSE: PhD Researcher, Strathclyde Law School, University of Strathclyde Glasgow United Kingdom: https://openalex.org/I181647926: University of Strathclyde: https://ror.org/00n3w3b69: GB: education: https://openalex.org/I181647926; https://openalex.org/A5071843257: Elisa Morgera: https://orcid.org/0000-0002-5234-8784: last: FALSE: Director, GCRF UKRI One Ocean Hub: https://openalex.org/I181647926: University of Strathclyde: https://ror.org/00n3w3b69: GB: education: https://openalex.org/I181647926</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Abstract After over a decade of international efforts to include the ocean in the policy discussions at the United Nations Framework Convention on Climate Change ( UNFCCC ) annual Conference of the Parties ( COP ), the ocean has finally been included by, inter alia , a reference to ‘ocean-based action’ in a series of COP outcomes, notable among which is the cover decisions known as the ‘Glasgow Climate Pact’. This article provides the necessary background to the inclusion of the ocean in COP 26 outcomes, including the Pact, and examines key issues, impacts and shortfalls of the Pact and other COP 26 outcomes, including mitigation, adaptation, finance and human rights. It concludes with suggestions for priority research areas moving forward.</t>
@@ -667,15 +655,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
+      <c r="T2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U2" t="b">
+        <v>1</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -687,41 +671,25 @@
           <t>https://brill.com/downloadpdf/journals/estu/37/1/article-p137_6.pdf</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
+      <c r="X2" t="b">
+        <v>1</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2024: 2023: 2022: 30: 19: 9</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
+      <c r="AA2">
+        <v>58</v>
+      </c>
+      <c r="AC2">
+        <v>2022</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>https://api.openalex.org/works?filter=cites:W4210835162</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W4210835162: https://doi.org/10.1163/15718085-bja10083</t>
-        </is>
-      </c>
       <c r="AF2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1163/15718085-bja10083</t>
@@ -732,52 +700,28 @@
           <t>article</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W2980737502</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>https://openalex.org/W4233921916: https://openalex.org/W3148144928: https://openalex.org/W2575112651: https://openalex.org/W235433852: https://openalex.org/W2119377653: https://openalex.org/W2068081422: https://openalex.org/W2020757966: https://openalex.org/W2005847371: https://openalex.org/W187456812: https://openalex.org/W1615167197</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>https://openalex.org/C2779073994: https://openalex.org/C17744445: https://openalex.org/C2780608745: https://openalex.org/C132651083: https://openalex.org/C2778539042: https://openalex.org/C199539241: https://openalex.org/C99743013: https://openalex.org/C111368507: https://openalex.org/C127313418: https://www.wikidata.org/wiki/Q1751686: https://www.wikidata.org/wiki/Q36442: https://www.wikidata.org/wiki/Q367293: https://www.wikidata.org/wiki/Q7942: https://www.wikidata.org/wiki/Q208645: https://www.wikidata.org/wiki/Q7748: https://www.wikidata.org/wiki/Q47359: https://www.wikidata.org/wiki/Q43518: https://www.wikidata.org/wiki/Q1069: Pact: Political science: Convention: Climate change: United Nations Framework Convention on Climate Change: Law: Kyoto Protocol: Oceanography: Geology: 2: 0: 2: 2: 4: 1: 3: 1: 0: 0.68293977: 0.58795327: 0.5614837: 0.50553393: 0.50141287: 0.18397388: 0.11712614: 0.11092797: 0</t>
-        </is>
+      <c r="AJ2" t="b">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="b">
+        <v>0</v>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>1: 0.9507: topic: https://openalex.org/T12414: Coastal and Marine Management; 1: 0.9507: subfield: https://openalex.org/subfields/2308: Management, Monitoring, Policy and Law; 1: 0.9507: field: https://openalex.org/fields/23: Environmental Science; 1: 0.9507: domain: https://openalex.org/domains/3: Physical Sciences</t>
+          <t>Coastal and Marine Management</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>Coastal and Marine Management</t>
+          <t>Management, Monitoring, Policy and Law</t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>Management, Monitoring, Policy and Law</t>
+          <t>Environmental Science</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
-        <is>
-          <t>Environmental Science</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
         <is>
           <t>Physical Sciences</t>
         </is>

</xml_diff>

<commit_message>
Revert "handling author complex data structure"
This reverts commit 29e46d208f80eee8cb30de9ce6817dda8949e2cd.
</commit_message>
<xml_diff>
--- a/citations/test_df.xlsx
+++ b/citations/test_df.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP2"/>
+  <dimension ref="A1:AQ2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -547,28 +547,35 @@
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
+          <t>topics</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
           <t>topic</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>subfield</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>2023</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -585,6 +592,11 @@
           <t>The Glasgow Climate Conference (COP26)</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://openalex.org/A5087355631: Mitchell Lennan: https://orcid.org/0000-0003-4744-4496: first: FALSE: PhD Researcher, Strathclyde Law School, University of Strathclyde Glasgow United Kingdom: https://openalex.org/I181647926: University of Strathclyde: https://ror.org/00n3w3b69: GB: education: https://openalex.org/I181647926; https://openalex.org/A5071843257: Elisa Morgera: https://orcid.org/0000-0002-5234-8784: last: FALSE: Director, GCRF UKRI One Ocean Hub: https://openalex.org/I181647926: University of Strathclyde: https://ror.org/00n3w3b69: GB: education: https://openalex.org/I181647926</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>Abstract After over a decade of international efforts to include the ocean in the policy discussions at the United Nations Framework Convention on Climate Change ( UNFCCC ) annual Conference of the Parties ( COP ), the ocean has finally been included by, inter alia , a reference to ‘ocean-based action’ in a series of COP outcomes, notable among which is the cover decisions known as the ‘Glasgow Climate Pact’. This article provides the necessary background to the inclusion of the ocean in COP 26 outcomes, including the Pact, and examines key issues, impacts and shortfalls of the Pact and other COP 26 outcomes, including mitigation, adaptation, finance and human rights. It concludes with suggestions for priority research areas moving forward.</t>
@@ -655,11 +667,15 @@
           <t>1</t>
         </is>
       </c>
-      <c r="T2" t="b">
-        <v>1</v>
-      </c>
-      <c r="U2" t="b">
-        <v>1</v>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -671,25 +687,41 @@
           <t>https://brill.com/downloadpdf/journals/estu/37/1/article-p137_6.pdf</t>
         </is>
       </c>
-      <c r="X2" t="b">
-        <v>1</v>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="AA2">
-        <v>58</v>
-      </c>
-      <c r="AC2">
-        <v>2022</v>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>2024: 2023: 2022: 30: 19: 9</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
           <t>https://api.openalex.org/works?filter=cites:W4210835162</t>
         </is>
       </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W4210835162: https://doi.org/10.1163/15718085-bja10083</t>
+        </is>
+      </c>
       <c r="AF2" t="inlineStr">
         <is>
           <t>https://doi.org/10.1163/15718085-bja10083</t>
@@ -700,28 +732,52 @@
           <t>article</t>
         </is>
       </c>
-      <c r="AJ2" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="b">
-        <v>0</v>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W2980737502</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>https://openalex.org/W4233921916: https://openalex.org/W3148144928: https://openalex.org/W2575112651: https://openalex.org/W235433852: https://openalex.org/W2119377653: https://openalex.org/W2068081422: https://openalex.org/W2020757966: https://openalex.org/W2005847371: https://openalex.org/W187456812: https://openalex.org/W1615167197</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>https://openalex.org/C2779073994: https://openalex.org/C17744445: https://openalex.org/C2780608745: https://openalex.org/C132651083: https://openalex.org/C2778539042: https://openalex.org/C199539241: https://openalex.org/C99743013: https://openalex.org/C111368507: https://openalex.org/C127313418: https://www.wikidata.org/wiki/Q1751686: https://www.wikidata.org/wiki/Q36442: https://www.wikidata.org/wiki/Q367293: https://www.wikidata.org/wiki/Q7942: https://www.wikidata.org/wiki/Q208645: https://www.wikidata.org/wiki/Q7748: https://www.wikidata.org/wiki/Q47359: https://www.wikidata.org/wiki/Q43518: https://www.wikidata.org/wiki/Q1069: Pact: Political science: Convention: Climate change: United Nations Framework Convention on Climate Change: Law: Kyoto Protocol: Oceanography: Geology: 2: 0: 2: 2: 4: 1: 3: 1: 0: 0.68293977: 0.58795327: 0.5614837: 0.50553393: 0.50141287: 0.18397388: 0.11712614: 0.11092797: 0</t>
+        </is>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
+          <t>1: 0.9507: topic: https://openalex.org/T12414: Coastal and Marine Management; 1: 0.9507: subfield: https://openalex.org/subfields/2308: Management, Monitoring, Policy and Law; 1: 0.9507: field: https://openalex.org/fields/23: Environmental Science; 1: 0.9507: domain: https://openalex.org/domains/3: Physical Sciences</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
           <t>Coastal and Marine Management</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>Management, Monitoring, Policy and Law</t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>Environmental Science</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>Physical Sciences</t>
         </is>

</xml_diff>